<commit_message>
Update requirements. Add USB connector and secure UART with pullups, fuse USB, UART and debugger pinout with TVS, fuse power lines with PTC and ceramic fuses (LLR_HW_1:LLR_HW_4; LLR_HW_16:LLR_HW_18).
</commit_message>
<xml_diff>
--- a/LED_Driver/LED Driver BOM.xlsx
+++ b/LED_Driver/LED Driver BOM.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Logic" sheetId="1" r:id="rId4"/>
+    <sheet state="visible" name="All" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="60">
   <si>
     <t>Symbol on schematic</t>
   </si>
@@ -35,13 +35,169 @@
   </si>
   <si>
     <t>https://www.tme.eu/pl/details/8.00m-smdhc49s/rezonatory-kwarcowe-smd/yic/</t>
+  </si>
+  <si>
+    <t>C1:C6</t>
+  </si>
+  <si>
+    <t>C1206 package 100nF capacitor</t>
+  </si>
+  <si>
+    <t>Noise reduction on supply lines</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>C8; C7</t>
+  </si>
+  <si>
+    <t>C1206 package 27pF capacitor</t>
+  </si>
+  <si>
+    <t>X1 load capacitors</t>
+  </si>
+  <si>
+    <t>R1; R2</t>
+  </si>
+  <si>
+    <t>R1206 package 100k resistor</t>
+  </si>
+  <si>
+    <t>Pull-up for reset and pull-down for BOOT mode</t>
+  </si>
+  <si>
+    <t>U1</t>
+  </si>
+  <si>
+    <t>STM32L152RET6</t>
+  </si>
+  <si>
+    <t>Main microcontroller</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/pl/details/stm32l152ret6/mikrokontrolery-st/stmicroelectronics/</t>
+  </si>
+  <si>
+    <t>SW1</t>
+  </si>
+  <si>
+    <t>THT tact switch</t>
+  </si>
+  <si>
+    <t>Reset switch, not mounted on real board.</t>
+  </si>
+  <si>
+    <t>U3</t>
+  </si>
+  <si>
+    <t>2.54 goldpin row, 5 pins</t>
+  </si>
+  <si>
+    <t>Programmer and debugger access.</t>
+  </si>
+  <si>
+    <t>USB1</t>
+  </si>
+  <si>
+    <t>ZX62D-B-5PA8(30)</t>
+  </si>
+  <si>
+    <t>USBC socket, communication.</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/pl/details/zx62d-b-5pa8-30/zlacza-usb-i-ieee1394/hirose/zx62d-b-5pa8-30/</t>
+  </si>
+  <si>
+    <t>R3</t>
+  </si>
+  <si>
+    <t>R1206 package 1.5k resistor</t>
+  </si>
+  <si>
+    <t>USB Data + pullup.</t>
+  </si>
+  <si>
+    <t>R4:R7</t>
+  </si>
+  <si>
+    <t>R1206 package resistors</t>
+  </si>
+  <si>
+    <t>Pullups and current limit on UART lines for safety concerns.</t>
+  </si>
+  <si>
+    <t>D1:D8</t>
+  </si>
+  <si>
+    <t>UCLAMP3301D</t>
+  </si>
+  <si>
+    <t>TVS diode for ESD protection</t>
+  </si>
+  <si>
+    <t>U2</t>
+  </si>
+  <si>
+    <t>2.54 goldpin row, 3 pins</t>
+  </si>
+  <si>
+    <t>UART vs. USB port selection</t>
+  </si>
+  <si>
+    <t>C9</t>
+  </si>
+  <si>
+    <t>Noise reduction on jumper line</t>
+  </si>
+  <si>
+    <t>F3</t>
+  </si>
+  <si>
+    <t>RF2643-000</t>
+  </si>
+  <si>
+    <t>5A PTC fuse</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/pl/details/ruef500/bezpieczniki-polimerowe-tht/littelfuse/rf2643-000/</t>
+  </si>
+  <si>
+    <t>F1</t>
+  </si>
+  <si>
+    <t>0ZCJ0020FF2E</t>
+  </si>
+  <si>
+    <t>0.2A PTC fuse</t>
+  </si>
+  <si>
+    <t>F2</t>
+  </si>
+  <si>
+    <t>PTS12066V100</t>
+  </si>
+  <si>
+    <t>1A PTC fuse</t>
+  </si>
+  <si>
+    <t>F4</t>
+  </si>
+  <si>
+    <t>0501020.WRS</t>
+  </si>
+  <si>
+    <t>20A fuse</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/pl/details/0501020.wr/bezpieczniki-smd-1206-szybkie/littelfuse/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -57,6 +213,10 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
     </font>
     <font>
       <u/>
@@ -83,7 +243,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -97,6 +257,9 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -315,7 +478,7 @@
     <col customWidth="1" min="1" max="1" width="16.88"/>
     <col customWidth="1" min="2" max="2" width="30.25"/>
     <col customWidth="1" min="3" max="3" width="51.38"/>
-    <col customWidth="1" min="4" max="4" width="58.5"/>
+    <col customWidth="1" min="4" max="4" width="61.25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -346,10 +509,211 @@
         <v>7</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="D2"/>
+    <hyperlink r:id="rId2" ref="D6"/>
+    <hyperlink r:id="rId3" ref="D9"/>
+    <hyperlink r:id="rId4" ref="D15"/>
+    <hyperlink r:id="rId5" ref="D18"/>
   </hyperlinks>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add PTC fuse in order to comply with LLR_HW_14 and LLR_HW_15. Research on OVP methods (see references).
</commit_message>
<xml_diff>
--- a/LED_Driver/LED Driver BOM.xlsx
+++ b/LED_Driver/LED Driver BOM.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="61">
   <si>
     <t>Symbol on schematic</t>
   </si>
@@ -191,6 +191,9 @@
   </si>
   <si>
     <t>https://www.tme.eu/pl/details/0501020.wr/bezpieczniki-smd-1206-szybkie/littelfuse/</t>
+  </si>
+  <si>
+    <t>F5</t>
   </si>
 </sst>
 </file>
@@ -706,6 +709,20 @@
         <v>59</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="D2"/>
@@ -713,7 +730,8 @@
     <hyperlink r:id="rId3" ref="D9"/>
     <hyperlink r:id="rId4" ref="D15"/>
     <hyperlink r:id="rId5" ref="D18"/>
+    <hyperlink r:id="rId6" ref="D19"/>
   </hyperlinks>
-  <drawing r:id="rId6"/>
+  <drawing r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>